<commit_message>
Add import_transactions.py to import project transactions from Excel
</commit_message>
<xml_diff>
--- a/Clints Sheet 12-05-2026.xlsx
+++ b/Clints Sheet 12-05-2026.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C7D7AA-E2FA-4523-995B-8C7D7F5EC42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3EA7EC67-EB00-450E-AA75-F0005FE37B45}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3EA7EC67-EB00-450E-AA75-F0005FE37B45}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="21" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2502,7 +2502,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2563,196 +2563,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{F749177F-CD5C-4A09-9496-02F758C55C95}"/>
   </cellStyles>
-  <dxfs count="95">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
+  <dxfs count="35">
     <dxf>
       <alignment vertical="center"/>
     </dxf>
@@ -12400,7 +12216,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B7FEC6A1-AE9E-4B6C-90DF-84B47A60FF29}" name="PivotTable1" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B7FEC6A1-AE9E-4B6C-90DF-84B47A60FF29}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
   <location ref="A1:C11" firstHeaderRow="2" firstDataRow="2" firstDataCol="2"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -12483,32 +12299,32 @@
     <dataField name="Count of تاريخ" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="20">
-    <format dxfId="79">
+    <format dxfId="19">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="78">
+    <format dxfId="18">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="17">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="16">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="15">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="72">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="0" count="1" selected="0">
@@ -12520,7 +12336,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="0" count="1" selected="0">
@@ -12532,35 +12348,35 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="70">
+    <format dxfId="10">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="69">
+    <format dxfId="9">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="8">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="7">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="6">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="5">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
     </format>
-    <format dxfId="64">
+    <format dxfId="4">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="0" count="1" selected="0">
@@ -12572,7 +12388,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="0" count="1" selected="0">
@@ -12584,7 +12400,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="0">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -12601,7 +12417,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D64D9B6B-CFC3-4674-8868-5BA6698C11A3}" name="PivotTable2" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D64D9B6B-CFC3-4674-8868-5BA6698C11A3}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
   <location ref="A1:C57" firstHeaderRow="2" firstDataRow="2" firstDataCol="2"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
@@ -12891,19 +12707,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{01D57055-2F68-4A21-BA36-E5D2385336C8}" name="Table1" displayName="Table1" ref="A1:J740" totalsRowShown="0" headerRowDxfId="94" dataDxfId="92" headerRowBorderDxfId="93" tableBorderDxfId="91" totalsRowBorderDxfId="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{01D57055-2F68-4A21-BA36-E5D2385336C8}" name="Table1" displayName="Table1" ref="A1:J740" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
   <autoFilter ref="A1:J740" xr:uid="{011C0CE7-6445-49C9-BBEE-21958062B1E4}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{15DAE80A-CB18-47F5-9E9F-207B5CEA88FE}" name="العميل" dataDxfId="89"/>
-    <tableColumn id="2" xr3:uid="{F9B6E543-5FF1-4370-918B-1FE2B6AA5C88}" name="المشروع" dataDxfId="88"/>
-    <tableColumn id="10" xr3:uid="{07CD6D2B-1DA7-4F23-BA72-CD067F0159C2}" name="إيرادات / مصروفات" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{7C63A4F0-5DD5-408C-8243-D2043EB77A3B}" name="تاريخ" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{92033B3D-6B32-4F3B-9A82-6C3A9714F901}" name="القسم" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{AC2088E6-82A2-4C45-B4F7-DE09BC175513}" name="البند تفصيلي" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{3FCBFE11-AD15-4F30-B723-37E3D169D704}" name="البيان" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{80818F4A-5EC6-4A91-93FA-1BA205D8E158}" name="منصرف" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{B352314C-04DA-4AD1-B27D-1A264AA4FFD7}" name="وارد" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{FBEBB221-129C-42E5-9C7B-5CD7285D281D}" name="نسبة الاشراف" dataDxfId="80"/>
+    <tableColumn id="1" xr3:uid="{15DAE80A-CB18-47F5-9E9F-207B5CEA88FE}" name="العميل" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{F9B6E543-5FF1-4370-918B-1FE2B6AA5C88}" name="المشروع" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{07CD6D2B-1DA7-4F23-BA72-CD067F0159C2}" name="إيرادات / مصروفات" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{7C63A4F0-5DD5-408C-8243-D2043EB77A3B}" name="تاريخ" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{92033B3D-6B32-4F3B-9A82-6C3A9714F901}" name="القسم" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{AC2088E6-82A2-4C45-B4F7-DE09BC175513}" name="البند تفصيلي" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{3FCBFE11-AD15-4F30-B723-37E3D169D704}" name="البيان" dataDxfId="23"/>
+    <tableColumn id="7" xr3:uid="{80818F4A-5EC6-4A91-93FA-1BA205D8E158}" name="منصرف" dataDxfId="22"/>
+    <tableColumn id="8" xr3:uid="{B352314C-04DA-4AD1-B27D-1A264AA4FFD7}" name="وارد" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{FBEBB221-129C-42E5-9C7B-5CD7285D281D}" name="نسبة الاشراف" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -35540,7 +35356,7 @@
       <c r="B3" s="2" t="s">
         <v>740</v>
       </c>
-      <c r="C3" s="23">
+      <c r="C3" s="2">
         <v>71</v>
       </c>
     </row>
@@ -35551,7 +35367,7 @@
       <c r="B4" s="2" t="s">
         <v>740</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C4" s="2">
         <v>595</v>
       </c>
     </row>
@@ -35562,7 +35378,7 @@
       <c r="B5" s="2" t="s">
         <v>742</v>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="2">
         <v>34</v>
       </c>
     </row>
@@ -35573,7 +35389,7 @@
       <c r="B6" s="2" t="s">
         <v>743</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="2">
         <v>4</v>
       </c>
     </row>
@@ -35584,7 +35400,7 @@
       <c r="B7" s="2" t="s">
         <v>745</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="2">
         <v>17</v>
       </c>
     </row>
@@ -35595,7 +35411,7 @@
       <c r="B8" s="2" t="s">
         <v>746</v>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="2">
         <v>8</v>
       </c>
     </row>
@@ -35606,7 +35422,7 @@
       <c r="B9" s="2" t="s">
         <v>709</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="2">
         <v>3</v>
       </c>
     </row>
@@ -35617,7 +35433,7 @@
       <c r="B10" s="2" t="s">
         <v>740</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="2">
         <v>7</v>
       </c>
     </row>
@@ -35625,7 +35441,7 @@
       <c r="A11" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="2">
         <v>739</v>
       </c>
     </row>
@@ -35667,7 +35483,7 @@
       <c r="B3" t="s">
         <v>485</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3">
         <v>2</v>
       </c>
     </row>
@@ -35678,7 +35494,7 @@
       <c r="B4" t="s">
         <v>485</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4">
         <v>4</v>
       </c>
     </row>
@@ -35689,7 +35505,7 @@
       <c r="B5" t="s">
         <v>750</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5">
         <v>10</v>
       </c>
     </row>
@@ -35700,7 +35516,7 @@
       <c r="B6" t="s">
         <v>385</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6">
         <v>3</v>
       </c>
     </row>
@@ -35711,7 +35527,7 @@
       <c r="B7" t="s">
         <v>414</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7">
         <v>2</v>
       </c>
     </row>
@@ -35722,7 +35538,7 @@
       <c r="B8" t="s">
         <v>450</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8">
         <v>1</v>
       </c>
     </row>
@@ -35733,7 +35549,7 @@
       <c r="B9" t="s">
         <v>727</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9">
         <v>90</v>
       </c>
     </row>
@@ -35744,7 +35560,7 @@
       <c r="B10" t="s">
         <v>385</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10">
         <v>5</v>
       </c>
     </row>
@@ -35755,7 +35571,7 @@
       <c r="B11" t="s">
         <v>757</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11">
         <v>9</v>
       </c>
     </row>
@@ -35766,7 +35582,7 @@
       <c r="B12" t="s">
         <v>582</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12">
         <v>8</v>
       </c>
     </row>
@@ -35777,7 +35593,7 @@
       <c r="B13" t="s">
         <v>479</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13">
         <v>1</v>
       </c>
     </row>
@@ -35788,7 +35604,7 @@
       <c r="B14" t="s">
         <v>426</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14">
         <v>26</v>
       </c>
     </row>
@@ -35799,7 +35615,7 @@
       <c r="B15" t="s">
         <v>652</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15">
         <v>4</v>
       </c>
     </row>
@@ -35810,7 +35626,7 @@
       <c r="B16" t="s">
         <v>539</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16">
         <v>6</v>
       </c>
     </row>
@@ -35821,7 +35637,7 @@
       <c r="B17" t="s">
         <v>165</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17">
         <v>3</v>
       </c>
     </row>
@@ -35832,7 +35648,7 @@
       <c r="B18" t="s">
         <v>545</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18">
         <v>2</v>
       </c>
     </row>
@@ -35843,7 +35659,7 @@
       <c r="B19" t="s">
         <v>727</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C19">
         <v>71</v>
       </c>
     </row>
@@ -35854,7 +35670,7 @@
       <c r="B20" t="s">
         <v>146</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20">
         <v>3</v>
       </c>
     </row>
@@ -35865,7 +35681,7 @@
       <c r="B21" t="s">
         <v>149</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21">
         <v>8</v>
       </c>
     </row>
@@ -35876,7 +35692,7 @@
       <c r="B22" t="s">
         <v>653</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22">
         <v>31</v>
       </c>
     </row>
@@ -35887,7 +35703,7 @@
       <c r="B23" t="s">
         <v>113</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23">
         <v>11</v>
       </c>
     </row>
@@ -35898,7 +35714,7 @@
       <c r="B24" t="s">
         <v>195</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24">
         <v>16</v>
       </c>
     </row>
@@ -35909,7 +35725,7 @@
       <c r="B25" t="s">
         <v>385</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25">
         <v>14</v>
       </c>
     </row>
@@ -35920,7 +35736,7 @@
       <c r="B26" t="s">
         <v>446</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26">
         <v>6</v>
       </c>
     </row>
@@ -35931,7 +35747,7 @@
       <c r="B27" t="s">
         <v>635</v>
       </c>
-      <c r="C27" s="22">
+      <c r="C27">
         <v>17</v>
       </c>
     </row>
@@ -35942,7 +35758,7 @@
       <c r="B28" t="s">
         <v>50</v>
       </c>
-      <c r="C28" s="22">
+      <c r="C28">
         <v>16</v>
       </c>
     </row>
@@ -35953,7 +35769,7 @@
       <c r="B29" t="s">
         <v>415</v>
       </c>
-      <c r="C29" s="22">
+      <c r="C29">
         <v>6</v>
       </c>
     </row>
@@ -35964,7 +35780,7 @@
       <c r="B30" t="s">
         <v>59</v>
       </c>
-      <c r="C30" s="22">
+      <c r="C30">
         <v>7</v>
       </c>
     </row>
@@ -35975,7 +35791,7 @@
       <c r="B31" t="s">
         <v>621</v>
       </c>
-      <c r="C31" s="22">
+      <c r="C31">
         <v>1</v>
       </c>
     </row>
@@ -35986,7 +35802,7 @@
       <c r="B32" t="s">
         <v>414</v>
       </c>
-      <c r="C32" s="22">
+      <c r="C32">
         <v>30</v>
       </c>
     </row>
@@ -35997,7 +35813,7 @@
       <c r="B33" t="s">
         <v>94</v>
       </c>
-      <c r="C33" s="22">
+      <c r="C33">
         <v>24</v>
       </c>
     </row>
@@ -36008,7 +35824,7 @@
       <c r="B34" t="s">
         <v>725</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34">
         <v>2</v>
       </c>
     </row>
@@ -36019,7 +35835,7 @@
       <c r="B35" t="s">
         <v>465</v>
       </c>
-      <c r="C35" s="22">
+      <c r="C35">
         <v>27</v>
       </c>
     </row>
@@ -36030,7 +35846,7 @@
       <c r="B36" t="s">
         <v>438</v>
       </c>
-      <c r="C36" s="22">
+      <c r="C36">
         <v>29</v>
       </c>
     </row>
@@ -36041,7 +35857,7 @@
       <c r="B37" t="s">
         <v>546</v>
       </c>
-      <c r="C37" s="22">
+      <c r="C37">
         <v>6</v>
       </c>
     </row>
@@ -36052,7 +35868,7 @@
       <c r="B38" t="s">
         <v>717</v>
       </c>
-      <c r="C38" s="22">
+      <c r="C38">
         <v>20</v>
       </c>
     </row>
@@ -36063,7 +35879,7 @@
       <c r="B39" t="s">
         <v>450</v>
       </c>
-      <c r="C39" s="22">
+      <c r="C39">
         <v>12</v>
       </c>
     </row>
@@ -36074,7 +35890,7 @@
       <c r="B40" t="s">
         <v>437</v>
       </c>
-      <c r="C40" s="22">
+      <c r="C40">
         <v>5</v>
       </c>
     </row>
@@ -36085,7 +35901,7 @@
       <c r="B41" t="s">
         <v>647</v>
       </c>
-      <c r="C41" s="22">
+      <c r="C41">
         <v>6</v>
       </c>
     </row>
@@ -36096,7 +35912,7 @@
       <c r="B42" t="s">
         <v>516</v>
       </c>
-      <c r="C42" s="22">
+      <c r="C42">
         <v>2</v>
       </c>
     </row>
@@ -36107,7 +35923,7 @@
       <c r="B43" t="s">
         <v>478</v>
       </c>
-      <c r="C43" s="22">
+      <c r="C43">
         <v>7</v>
       </c>
     </row>
@@ -36118,7 +35934,7 @@
       <c r="B44" t="s">
         <v>25</v>
       </c>
-      <c r="C44" s="22">
+      <c r="C44">
         <v>12</v>
       </c>
     </row>
@@ -36129,7 +35945,7 @@
       <c r="B45" t="s">
         <v>594</v>
       </c>
-      <c r="C45" s="22">
+      <c r="C45">
         <v>2</v>
       </c>
     </row>
@@ -36140,7 +35956,7 @@
       <c r="B46" t="s">
         <v>523</v>
       </c>
-      <c r="C46" s="22">
+      <c r="C46">
         <v>6</v>
       </c>
     </row>
@@ -36151,7 +35967,7 @@
       <c r="B47" t="s">
         <v>532</v>
       </c>
-      <c r="C47" s="22">
+      <c r="C47">
         <v>1</v>
       </c>
     </row>
@@ -36162,7 +35978,7 @@
       <c r="B48" t="s">
         <v>464</v>
       </c>
-      <c r="C48" s="22">
+      <c r="C48">
         <v>40</v>
       </c>
     </row>
@@ -36173,7 +35989,7 @@
       <c r="B49" t="s">
         <v>751</v>
       </c>
-      <c r="C49" s="22">
+      <c r="C49">
         <v>18</v>
       </c>
     </row>
@@ -36184,7 +36000,7 @@
       <c r="B50" t="s">
         <v>752</v>
       </c>
-      <c r="C50" s="22">
+      <c r="C50">
         <v>18</v>
       </c>
     </row>
@@ -36195,7 +36011,7 @@
       <c r="B51" t="s">
         <v>753</v>
       </c>
-      <c r="C51" s="22">
+      <c r="C51">
         <v>6</v>
       </c>
     </row>
@@ -36206,7 +36022,7 @@
       <c r="B52" t="s">
         <v>754</v>
       </c>
-      <c r="C52" s="22">
+      <c r="C52">
         <v>16</v>
       </c>
     </row>
@@ -36217,7 +36033,7 @@
       <c r="B53" t="s">
         <v>755</v>
       </c>
-      <c r="C53" s="22">
+      <c r="C53">
         <v>4</v>
       </c>
     </row>
@@ -36228,7 +36044,7 @@
       <c r="B54" t="s">
         <v>756</v>
       </c>
-      <c r="C54" s="22">
+      <c r="C54">
         <v>2</v>
       </c>
     </row>
@@ -36239,7 +36055,7 @@
       <c r="B55" t="s">
         <v>758</v>
       </c>
-      <c r="C55" s="22">
+      <c r="C55">
         <v>1</v>
       </c>
     </row>
@@ -36250,7 +36066,7 @@
       <c r="B56" t="s">
         <v>759</v>
       </c>
-      <c r="C56" s="22">
+      <c r="C56">
         <v>3</v>
       </c>
     </row>
@@ -36258,7 +36074,7 @@
       <c r="A57" t="s">
         <v>343</v>
       </c>
-      <c r="C57" s="22">
+      <c r="C57">
         <v>682</v>
       </c>
     </row>

</xml_diff>